<commit_message>
Test plan: note how the Summary counts behave
The Summary sheet's counts are live COUNTA/COUNTIF formulas written without
cached values, so Excel computes them on open but a preview tool may show them
blank. Said so on the Read me sheet rather than leaving it to be discovered.

Automated recalculation could not verify them here: LibreOffice does not run in
this container (a three-cell test file fails the same way), so recalc.py never
completed. The formulas were checked by inspection instead - every cross-sheet
reference resolves to a real sheet name, and the COUNTIF columns match the
Priority and Result headers on every suite sheet, which share one layout. Only
COUNTA, COUNTIF and SUM are used, all of which Excel and LibreOffice evaluate
without a prefix.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/freeitsm-test-plan-new-suites.xlsx
+++ b/freeitsm-test-plan-new-suites.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -646,6 +646,37 @@
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Fill in Result (Pass / Fail / Blocked / N-A), Tester and Notes as you go.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>A note on the Summary sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Its counts are live formulas (COUNTA / COUNTIF) over the suite sheets. They were written</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>without cached values, so Excel computes them the moment you open the file. If a preview tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>shows the Summary as blank or zero, open the workbook in Excel and the figures appear.</t>
         </is>
       </c>
     </row>

</xml_diff>